<commit_message>
Importers: master-data + BOM Excel -> Postgres (validated)
- scripts/_import_utils.py: row reader (skips blanks + leftover template example
  rows), Report (per-sheet counts + errors)
- scripts/import_master_data.py: WarehouseLocation/Supplier/Customer/Item/GlueRecipe
  (+components)/LogArrival/Log; auto-masters species; resolves supplier refs;
  dual-unit log fill; upsert + error report
- scripts/import_bom.py: Assembly_BOM -> Product (+ auto-mastered category) + rebuilt
  ASSEMBLY BOM lines (board/veneer=items, glue=recipe, coating/packing=items);
  Transform_PVS/PSP -> TransformationRecipe + lines; FK resolution + error report
- build_templates: drop inline example rows (data starts row 2); expose EXAMPLES
- Self-tested on a sample with deliberate errors: valid rows imported, bad kind /
  unknown refs reported and skipped; verified BOM structure in DB. Dev DB reset after.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/pvwood_master_data.xlsx
+++ b/templates/pvwood_master_data.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,10 +35,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
     </font>
     <font>
       <b val="1"/>
@@ -70,16 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -556,27 +551,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>WH-A1</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Warehouse A Rack 1</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>WAREHOUSE</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"WAREHOUSE,FC,WIP,FG,STAGING"</formula1>
     </dataValidation>
   </dataValidations>
@@ -590,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -639,31 +616,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>SUP001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>ACME Veneer Co</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>K. Somchai</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>0812345678</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -675,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -718,22 +670,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Global Doors Ltd</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>J. Smith</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -745,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -890,106 +826,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>VNR-OAK-CQ-A</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>VENEER</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Oak Crown A</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>OAK</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>CROWN</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>BOOK</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>FACE</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>FSC100</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>1270</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>5201</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>SUP001</t>
-        </is>
-      </c>
-      <c r="W2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B3:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"VENEER,BOARD,GLUE_COMPONENT,CONSUMABLE,PACKING,OTHER"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1003,7 +842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1064,49 +903,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>GL-STD</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Standard UF</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1118,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1149,28 +945,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>GL-STD</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>resin</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>GLU-UF-RESIN</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1182,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1219,29 +993,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>ARR-2026-001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>SUP001</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>MSKU1234567</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1253,7 +1004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1332,64 +1083,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>LOG-0001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>ARR-2026-001</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>OAK-A</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>OAK</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>98</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>0.61</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>photo in notes</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>